<commit_message>
Add README and test_plan file
</commit_message>
<xml_diff>
--- a/test_plan.xlsx
+++ b/test_plan.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
-  <workbookPr defaultThemeVersion="202300"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="20417"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\DV\APB2UART\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{03BE1877-84B2-4E16-BF90-E44699D8F152}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{202F65A7-3DE4-49E4-98F7-44341A9E9CB5}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{649ECBB2-2976-4DF4-88DC-386B70686C8C}"/>
   </bookViews>
@@ -20,23 +20,12 @@
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
     </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="40">
   <si>
     <t>LABEL</t>
   </si>
@@ -54,12 +43,6 @@
   </si>
   <si>
     <t>DESIGN REQUIREMENT DESCRIPTION</t>
-  </si>
-  <si>
-    <t>directed test at the beginning of the simulation then randomized with constraint that reset deasserted most of the time</t>
-  </si>
-  <si>
-    <t>define coverpoint of data register</t>
   </si>
   <si>
     <t>Compare actual data to ref model 
@@ -79,41 +62,69 @@
 bits in CONTROL register</t>
   </si>
   <si>
-    <t>UART_FRAME</t>
-  </si>
-  <si>
-    <t>UART Frame includes START, 8-bit DATA, 
-PARITY(optional) and STOP bits</t>
+    <t>randomize the value of DIVISOR register that
+only lies between those values</t>
+  </si>
+  <si>
+    <t>UART supports interrupt for parity_error, frame_error, 
+break condition, tx overrun, rx_overrun, rx_data (complete rx_data)</t>
+  </si>
+  <si>
+    <t>Checkers to track interrupt interface as HIGH level</t>
+  </si>
+  <si>
+    <t>UART_ERROR</t>
+  </si>
+  <si>
+    <t>When reset is active (low-level) CONTROL, STATUS, DIVISOR registers contain '0' value, TX FSM and RX FSM state are IDLE, TX FIFO and RX FIFO are EMPTY</t>
+  </si>
+  <si>
+    <t xml:space="preserve">directed test at the beginning of the simulation </t>
+  </si>
+  <si>
+    <t>Concurrent assertion to check (System Verilog bind)</t>
+  </si>
+  <si>
+    <t>NO PARITY</t>
+  </si>
+  <si>
+    <t>UART Frame includes START bit, 8-bit DATA, 
+and STOP bit</t>
+  </si>
+  <si>
+    <t>disable parity_en bit in CONTROL register
+randomize DATA</t>
+  </si>
+  <si>
+    <t>PARITY</t>
+  </si>
+  <si>
+    <t>UART Frame includes START bit, 8-bit DATA, 
+PARITY bit and STOP bit</t>
+  </si>
+  <si>
+    <t>define coverpoint of data register,
+define coverpoint of parity 
+use cross coverage with these two coverpoint</t>
   </si>
   <si>
     <t>randomize with constraints to generate a mix of even or odd bit-1 count (full bit 0, full bit 1,
 even bit 1, odd bit 1) of 8-bit DATA
-- randomize parity_en bit in CONTROL register with 60 (logic 1)/40 (logic 0) ratio</t>
-  </si>
-  <si>
-    <t>randomize the value of DIVISOR register that
-only lies between those values</t>
-  </si>
-  <si>
-    <t>UART supports interrupt for parity_error, frame_error, 
-break condition, tx overrun, rx_overrun, rx_data (complete rx_data)</t>
-  </si>
-  <si>
-    <t>As reset is active (low-level) CONTROL, STATUS, DIVISOR registers contain '0' value, TX FSM and RX FSM state are IDLE, TX FIFO and RX FIFO are EMPTY</t>
-  </si>
-  <si>
-    <t>Checkers to track interrupt interface as HIGH level</t>
-  </si>
-  <si>
-    <t>UART_ERROR</t>
-  </si>
-  <si>
-    <t>Frame error, parity error, break condition, tx overrun, 
-rx overrun</t>
-  </si>
-  <si>
-    <t>Checkers to count times of HIGH level of bits
-in STATUS register</t>
+- randomize parity_en bit in CONTROL register with 60 (logic 1)/40 (logic 0) ratio
+to configure odd parity and even parity</t>
+  </si>
+  <si>
+    <t>define coverpoint of divisor value</t>
+  </si>
+  <si>
+    <t>Fix array to contain name of all bits of STATUS register (1)
+Associative array to contain counter of each bit with index in (1) to track HIGH count of each bit</t>
+  </si>
+  <si>
+    <t>STATUS register</t>
+  </si>
+  <si>
+    <t>Frame error, parity error, break condition</t>
   </si>
   <si>
     <r>
@@ -123,6 +134,133 @@
         <color theme="1"/>
         <rFont val="Aptos Narrow"/>
         <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Frame error, parity error, break condition</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">: 
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="14"/>
+        <color theme="4"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Idea</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">: total cycles to sample full frame of UART1 is excess to total cycles of shifting START bit of UART0
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="14"/>
+        <color theme="4"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Set up</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>: UART0: 9600 (BRR = 324), UART1: 115200 (BRR = 26) and configure parity type is odd parity</t>
+    </r>
+  </si>
+  <si>
+    <t>define coverpoint of each error case</t>
+  </si>
+  <si>
+    <t>tx_full, rx_full, tx_overrun, rx_overrun, busy, rx_not_empty</t>
+  </si>
+  <si>
+    <t>define coverpoint of each bit</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">Directed Test:
+Idea:
+TX Full: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">Write 8 TX data to TX_FIFO and do not write DIVISOR value to hardware.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>RX Full</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">: Write 8 TX data to TX_FIFO and do not read RX_FIFO </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
         <scheme val="minor"/>
       </rPr>
       <t>TX overrun</t>
@@ -144,10 +282,9 @@
         <sz val="14"/>
         <color theme="1"/>
         <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Rx overrun</t>
+        <scheme val="minor"/>
+      </rPr>
+      <t>RX overrun</t>
     </r>
     <r>
       <rPr>
@@ -163,13 +300,48 @@
     <r>
       <rPr>
         <b/>
+        <u/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Note</t>
+    </r>
+    <r>
+      <rPr>
         <sz val="14"/>
         <color theme="1"/>
         <rFont val="Aptos Narrow"/>
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
-      <t>Frame error, parity error, break condition</t>
+      <t>: calculate the required clock cycles to read STATUS register in all cases</t>
+    </r>
+  </si>
+  <si>
+    <t>DIFFERENT 
+FREQUENCY</t>
+  </si>
+  <si>
+    <t>2 UART can communicate with two frequencies</t>
+  </si>
+  <si>
+    <t>Set two different frequencies for 2 UART</t>
+  </si>
+  <si>
+    <t>CONFIG WRITE ACCESS</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Reconfig</t>
     </r>
     <r>
       <rPr>
@@ -179,59 +351,39 @@
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
-      <t xml:space="preserve">: 
+      <t xml:space="preserve">: When UART starts, configuration that includes baud rate, parity enable, … can be reconfigured at suitable time (check BUSY bit in STATUS register before doing reconfiguration)
 </t>
     </r>
     <r>
       <rPr>
         <b/>
         <sz val="14"/>
-        <color theme="4"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Ignored</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <color theme="1"/>
         <rFont val="Aptos Narrow"/>
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
-      <t>Idea</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">: total cycles to sample full frame of UART1 is excess to total cycles of shifting START bit of UART0
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="14"/>
-        <color theme="4"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Set up</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>: UART0: 9600 (BRR = 324), UART1: 115200 (BRR = 26) and configure parity type is odd parity</t>
-    </r>
+      <t>: When UARTs, bit BUSY is HIGH, this write access is ignored</t>
+    </r>
+  </si>
+  <si>
+    <t>Write one TX_DATA, calculate the required time to read and check BUSY bit of STATUS register, do reconfig.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="8">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -269,6 +421,27 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="14"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="14"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <u/>
+      <sz val="14"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="3">
     <fill>
@@ -369,7 +542,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -388,6 +561,9 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -723,18 +899,18 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7DD4153B-7C4D-46B8-98F6-4C20189A1A48}">
-  <dimension ref="A1:E22"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:E26"/>
+  <sheetFormatPr defaultRowHeight="13.8"/>
   <cols>
-    <col min="1" max="1" width="18.5546875" customWidth="1"/>
-    <col min="2" max="2" width="55.6640625" customWidth="1"/>
-    <col min="3" max="3" width="46.5546875" customWidth="1"/>
-    <col min="4" max="4" width="35.109375" customWidth="1"/>
-    <col min="5" max="5" width="50.77734375" customWidth="1"/>
-    <col min="6" max="6" width="26.77734375" customWidth="1"/>
+    <col min="1" max="1" width="23.5" customWidth="1"/>
+    <col min="2" max="2" width="55.69921875" customWidth="1"/>
+    <col min="3" max="3" width="46.59765625" customWidth="1"/>
+    <col min="4" max="4" width="42.19921875" customWidth="1"/>
+    <col min="5" max="5" width="50.796875" customWidth="1"/>
+    <col min="6" max="6" width="26.796875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="24.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="1" spans="1:5" ht="24" thickTop="1" thickBot="1">
       <c r="A1" s="6" t="s">
         <v>0</v>
       </c>
@@ -751,191 +927,261 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:5" ht="71.400000000000006" customHeight="1" thickTop="1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:5" ht="71.400000000000006" customHeight="1" thickTop="1">
       <c r="A2" s="4" t="s">
         <v>4</v>
       </c>
       <c r="B2" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="C2" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="D2" s="4"/>
+      <c r="E2" s="5" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" ht="71.400000000000006" customHeight="1">
+      <c r="A3" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="C2" s="5" t="s">
+      <c r="B3" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="C3" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="D3" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="E3" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="D2" s="4"/>
-      <c r="E2" s="5"/>
-    </row>
-    <row r="3" spans="1:5" ht="106.2" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A3" s="1" t="s">
+    </row>
+    <row r="4" spans="1:5" ht="106.2" customHeight="1">
+      <c r="A4" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="E4" s="2" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" ht="47.4" customHeight="1">
+      <c r="A5" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="D5" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="E5" s="1"/>
+    </row>
+    <row r="6" spans="1:5" ht="121.2" customHeight="1">
+      <c r="A6" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="D6" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="E6" s="2" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" ht="138.6" customHeight="1">
+      <c r="A7" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="C7" s="9" t="s">
+        <v>33</v>
+      </c>
+      <c r="D7" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="E7" s="2" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" ht="73.8" customHeight="1">
+      <c r="A8" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="C8" s="9" t="s">
+        <v>36</v>
+      </c>
+      <c r="D8" s="1"/>
+      <c r="E8" s="2" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" ht="129" customHeight="1">
+      <c r="A9" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="B9" s="9" t="s">
+        <v>38</v>
+      </c>
+      <c r="C9" s="9" t="s">
+        <v>39</v>
+      </c>
+      <c r="D9" s="1"/>
+      <c r="E9" s="2" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" ht="69.599999999999994">
+      <c r="A10" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="D10" s="1"/>
+      <c r="E10" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="B3" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="C3" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="D3" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="E3" s="2" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5" ht="47.4" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A4" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="B4" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="C4" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="D4" s="1"/>
-      <c r="E4" s="1"/>
-    </row>
-    <row r="5" spans="1:5" ht="54" x14ac:dyDescent="0.35">
-      <c r="A5" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="B5" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="C5" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="D5" s="1"/>
-      <c r="E5" s="2" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5" ht="236.4" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A6" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="B6" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="C6" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="D6" s="1"/>
-      <c r="E6" s="2" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="7" spans="1:5" ht="18" x14ac:dyDescent="0.35">
-      <c r="A7" s="3"/>
-      <c r="B7" s="3"/>
-      <c r="C7" s="3"/>
-      <c r="D7" s="3"/>
-      <c r="E7" s="3"/>
-    </row>
-    <row r="8" spans="1:5" ht="18" x14ac:dyDescent="0.35">
-      <c r="A8" s="3"/>
-      <c r="B8" s="3"/>
-      <c r="C8" s="3"/>
-      <c r="D8" s="3"/>
-      <c r="E8" s="3"/>
-    </row>
-    <row r="9" spans="1:5" ht="18" x14ac:dyDescent="0.35">
-      <c r="A9" s="3"/>
-      <c r="B9" s="3"/>
-      <c r="C9" s="3"/>
-      <c r="D9" s="3"/>
-      <c r="E9" s="3"/>
-    </row>
-    <row r="10" spans="1:5" ht="18" x14ac:dyDescent="0.35">
-      <c r="A10" s="3"/>
-      <c r="B10" s="3"/>
-      <c r="C10" s="3"/>
-      <c r="D10" s="3"/>
-      <c r="E10" s="3"/>
-    </row>
-    <row r="11" spans="1:5" ht="18" x14ac:dyDescent="0.35">
+    </row>
+    <row r="11" spans="1:5" ht="17.399999999999999">
       <c r="A11" s="3"/>
       <c r="B11" s="3"/>
       <c r="C11" s="3"/>
       <c r="D11" s="3"/>
       <c r="E11" s="3"/>
     </row>
-    <row r="12" spans="1:5" ht="18" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:5" ht="17.399999999999999">
       <c r="A12" s="3"/>
       <c r="B12" s="3"/>
       <c r="C12" s="3"/>
       <c r="D12" s="3"/>
       <c r="E12" s="3"/>
     </row>
-    <row r="13" spans="1:5" ht="18" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:5" ht="17.399999999999999">
       <c r="A13" s="3"/>
       <c r="B13" s="3"/>
       <c r="C13" s="3"/>
       <c r="D13" s="3"/>
       <c r="E13" s="3"/>
     </row>
-    <row r="14" spans="1:5" ht="18" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:5" ht="17.399999999999999">
       <c r="A14" s="3"/>
       <c r="B14" s="3"/>
       <c r="C14" s="3"/>
       <c r="D14" s="3"/>
       <c r="E14" s="3"/>
     </row>
-    <row r="15" spans="1:5" ht="18" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:5" ht="17.399999999999999">
       <c r="A15" s="3"/>
       <c r="B15" s="3"/>
       <c r="C15" s="3"/>
       <c r="D15" s="3"/>
       <c r="E15" s="3"/>
     </row>
-    <row r="16" spans="1:5" ht="18" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:5" ht="17.399999999999999">
       <c r="A16" s="3"/>
       <c r="B16" s="3"/>
       <c r="C16" s="3"/>
       <c r="D16" s="3"/>
       <c r="E16" s="3"/>
     </row>
-    <row r="17" spans="1:5" ht="18" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:5" ht="17.399999999999999">
       <c r="A17" s="3"/>
       <c r="B17" s="3"/>
       <c r="C17" s="3"/>
       <c r="D17" s="3"/>
       <c r="E17" s="3"/>
     </row>
-    <row r="18" spans="1:5" ht="18" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:5" ht="17.399999999999999">
       <c r="A18" s="3"/>
       <c r="B18" s="3"/>
       <c r="C18" s="3"/>
       <c r="D18" s="3"/>
       <c r="E18" s="3"/>
     </row>
-    <row r="19" spans="1:5" ht="18" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:5" ht="17.399999999999999">
       <c r="A19" s="3"/>
       <c r="B19" s="3"/>
       <c r="C19" s="3"/>
       <c r="D19" s="3"/>
       <c r="E19" s="3"/>
     </row>
-    <row r="20" spans="1:5" ht="18" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:5" ht="17.399999999999999">
       <c r="A20" s="3"/>
       <c r="B20" s="3"/>
       <c r="C20" s="3"/>
       <c r="D20" s="3"/>
       <c r="E20" s="3"/>
     </row>
-    <row r="21" spans="1:5" ht="18" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:5" ht="17.399999999999999">
       <c r="A21" s="3"/>
       <c r="B21" s="3"/>
       <c r="C21" s="3"/>
       <c r="D21" s="3"/>
       <c r="E21" s="3"/>
     </row>
-    <row r="22" spans="1:5" ht="18" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:5" ht="17.399999999999999">
       <c r="A22" s="3"/>
       <c r="B22" s="3"/>
       <c r="C22" s="3"/>
       <c r="D22" s="3"/>
       <c r="E22" s="3"/>
     </row>
+    <row r="23" spans="1:5" ht="17.399999999999999">
+      <c r="A23" s="3"/>
+      <c r="B23" s="3"/>
+      <c r="C23" s="3"/>
+      <c r="D23" s="3"/>
+      <c r="E23" s="3"/>
+    </row>
+    <row r="24" spans="1:5" ht="17.399999999999999">
+      <c r="A24" s="3"/>
+      <c r="B24" s="3"/>
+      <c r="C24" s="3"/>
+      <c r="D24" s="3"/>
+      <c r="E24" s="3"/>
+    </row>
+    <row r="25" spans="1:5" ht="17.399999999999999">
+      <c r="A25" s="3"/>
+      <c r="B25" s="3"/>
+      <c r="C25" s="3"/>
+      <c r="D25" s="3"/>
+      <c r="E25" s="3"/>
+    </row>
+    <row r="26" spans="1:5" ht="17.399999999999999">
+      <c r="A26" s="3"/>
+      <c r="B26" s="3"/>
+      <c r="C26" s="3"/>
+      <c r="D26" s="3"/>
+      <c r="E26" s="3"/>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>